<commit_message>
feat: implement comprehensive invoice management, financial overview dashboard, and student/product features.
</commit_message>
<xml_diff>
--- a/public/files/Student-format.xlsx
+++ b/public/files/Student-format.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9264"/>
+    <workbookView windowWidth="23040" windowHeight="9707"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,12 +27,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>Roll Number</t>
+  </si>
   <si>
     <t>Name</t>
   </si>
   <si>
     <t>Admission Number</t>
+  </si>
+  <si>
+    <t>Balance</t>
   </si>
 </sst>
 </file>
@@ -660,7 +666,7 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
@@ -1185,15 +1191,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="3"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="3" max="3" width="17.7777777777778" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>